<commit_message>
vault backup: 2026-07-09 16:10:27
</commit_message>
<xml_diff>
--- a/areas/Workout log.xlsx
+++ b/areas/Workout log.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Date</t>
   </si>
@@ -75,6 +75,9 @@
   <si>
     <t xml:space="preserve">GTG (Greasing the groove) accessory workouts are done throughout the day without any strict rest time (&gt; 10 minutes)</t>
   </si>
+  <si>
+    <t>Rest</t>
+  </si>
 </sst>
 </file>
 
@@ -94,7 +97,7 @@
       <b/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -105,6 +108,12 @@
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.59999389629810485"/>
         <bgColor theme="6" tint="0.59999389629810485"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor theme="9" tint="0.59999389629810485"/>
       </patternFill>
     </fill>
   </fills>
@@ -134,10 +143,10 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf fontId="0" fillId="3" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1" quotePrefix="0" pivotButton="0">
+    <xf fontId="0" fillId="3" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
@@ -728,16 +737,16 @@
       <c r="C2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="5">
+      <c r="D2" s="4">
         <v>21</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E2" s="4">
         <v>18.800000000000001</v>
       </c>
-      <c r="F2" s="5">
+      <c r="F2" s="4">
         <v>60.799999999999997</v>
       </c>
-      <c r="G2" s="5">
+      <c r="G2" s="4">
         <v>8</v>
       </c>
       <c r="H2" s="4" t="s">
@@ -754,7 +763,7 @@
       <c r="C3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="1" t="s">
         <v>13</v>
       </c>
       <c r="E3" s="1">
@@ -774,13 +783,15 @@
       <c r="A4" s="3">
         <v>46211</v>
       </c>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
+      <c r="B4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
     </row>
     <row r="5" ht="14.25">
       <c r="A5" s="3">

</xml_diff>

<commit_message>
vault backup: 2026-07-10 22:28:33
</commit_message>
<xml_diff>
--- a/areas/Workout log.xlsx
+++ b/areas/Workout log.xlsx
@@ -129,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" quotePrefix="0" pivotButton="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="left" vertical="top"/>
@@ -142,9 +142,6 @@
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="3" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf fontId="0" fillId="3" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="left" vertical="top"/>
@@ -786,24 +783,26 @@
       <c r="B4" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
     </row>
     <row r="5" ht="14.25">
       <c r="A5" s="3">
         <v>46212</v>
       </c>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
+      <c r="B5" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
     </row>
     <row r="6" ht="14.25">
       <c r="A6" s="3">

</xml_diff>

<commit_message>
vault backup: 2026-07-13 12:53:02
</commit_message>
<xml_diff>
--- a/areas/Workout log.xlsx
+++ b/areas/Workout log.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>Date</t>
   </si>
@@ -78,6 +78,9 @@
   <si>
     <t>Rest</t>
   </si>
+  <si>
+    <t>Swim</t>
+  </si>
 </sst>
 </file>
 
@@ -129,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" quotePrefix="0" pivotButton="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="left" vertical="top"/>
@@ -143,7 +146,16 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf fontId="0" fillId="3" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf fontId="0" fillId="3" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
@@ -731,19 +743,19 @@
       <c r="B2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="5">
         <v>21</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E2" s="5">
         <v>18.800000000000001</v>
       </c>
-      <c r="F2" s="4">
+      <c r="F2" s="5">
         <v>60.799999999999997</v>
       </c>
-      <c r="G2" s="4">
+      <c r="G2" s="5">
         <v>8</v>
       </c>
       <c r="H2" s="4" t="s">
@@ -757,7 +769,7 @@
       <c r="B3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="5" t="s">
         <v>12</v>
       </c>
       <c r="D3" s="1" t="s">
@@ -772,7 +784,7 @@
       <c r="G3" s="1">
         <v>8.5</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="5" t="s">
         <v>14</v>
       </c>
     </row>
@@ -780,35 +792,37 @@
       <c r="A4" s="3">
         <v>46211</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
     </row>
     <row r="5" ht="14.25">
       <c r="A5" s="3">
         <v>46212</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
     </row>
     <row r="6" ht="14.25">
       <c r="A6" s="3">
         <v>46213</v>
       </c>
-      <c r="B6" s="1"/>
+      <c r="B6" s="8" t="s">
+        <v>16</v>
+      </c>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
@@ -820,13 +834,15 @@
       <c r="A7" s="3">
         <v>46214</v>
       </c>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
+      <c r="B7" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
     </row>
     <row r="8" ht="14.25">
       <c r="A8" s="3">

</xml_diff>